<commit_message>
Retry Failed Testcases Login Added
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/09_MyWebSite/MyWebSite/01_MyWebSiteTest.xlsx
+++ b/src/test/resources/testdata/Modules/09_MyWebSite/MyWebSite/01_MyWebSiteTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\09_MyWebSite\MyWebSite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94E7885B-F409-4A0E-A07E-E76A296513A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BECD1804-3F8A-446B-B703-7D5FC92AE473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2260" uniqueCount="559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2260" uniqueCount="560">
   <si>
     <t>TESTCASE_ID</t>
   </si>
@@ -10632,6 +10632,12 @@
 hidekeyboard
 clickon_nextbtn
 clickon_nextbtn
+verify_alert_dialog_title</t>
+  </si>
+  <si>
+    <t>project_add_projects
+project_clickon_submitbtn
+project_clickon_submitbtn
 verify_alert_dialog_title</t>
   </si>
 </sst>
@@ -15956,7 +15962,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="141" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:14" ht="58" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>8</v>
       </c>
@@ -15970,7 +15976,7 @@
         <v>265</v>
       </c>
       <c r="E141" s="6" t="s">
-        <v>524</v>
+        <v>559</v>
       </c>
       <c r="F141" s="1"/>
       <c r="G141" s="1"/>

</xml_diff>